<commit_message>
some changes done in excel
</commit_message>
<xml_diff>
--- a/TestPlane_Task2_25MCMT38.xlsx
+++ b/TestPlane_Task2_25MCMT38.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/33811ab4aed103c6/OD_Developer_WordFiles/MtechNotes/Sem2/SE_and_SE_Lab/SRPS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A05ACBEF-7EAB-5D43-80E1-A8581DFD61F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{A05ACBEF-7EAB-5D43-80E1-A8581DFD61F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21BCCD25-2EE9-474F-91D2-C7A3C84EC4AB}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{749BA49F-03DC-3D4A-8A5F-ADEAC108BE1C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17280" xr2:uid="{749BA49F-03DC-3D4A-8A5F-ADEAC108BE1C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
     <t>Project Name</t>
   </si>
   <si>
-    <t>Student Registration System (SRPS)</t>
-  </si>
-  <si>
     <t>Browser:</t>
   </si>
   <si>
@@ -189,6 +186,9 @@
   </si>
   <si>
     <t>Pass</t>
+  </si>
+  <si>
+    <t>Student Result Processing  System (SRPS)</t>
   </si>
 </sst>
 </file>
@@ -298,6 +298,13 @@
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -307,19 +314,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,372 +668,372 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="6"/>
+      <c r="G2" s="9"/>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="9"/>
     </row>
     <row r="4" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="6"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="7">
-        <v>46043</v>
-      </c>
-      <c r="G5" s="6"/>
+      <c r="F5" s="8">
+        <v>46043</v>
+      </c>
+      <c r="G5" s="9"/>
     </row>
     <row r="8" spans="1:7" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="G8" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="4">
         <v>46043</v>
       </c>
       <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
-        <v>23</v>
-      </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="4">
         <v>46043</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" t="s">
         <v>24</v>
       </c>
-      <c r="E10" t="s">
-        <v>25</v>
-      </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>3</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="4">
         <v>46043</v>
       </c>
       <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
         <v>26</v>
       </c>
-      <c r="D11" t="s">
-        <v>27</v>
-      </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="4">
         <v>46043</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>5</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="4">
         <v>46043</v>
       </c>
       <c r="C13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" t="s">
-        <v>30</v>
-      </c>
       <c r="E13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>6</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="4">
         <v>46043</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>7</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="4">
         <v>46043</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D15">
         <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>8</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="4">
         <v>46043</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D16">
         <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>9</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="4">
         <v>46043</v>
       </c>
       <c r="C17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s">
         <v>35</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>36</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>37</v>
       </c>
-      <c r="F17" t="s">
-        <v>38</v>
-      </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>10</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="4">
         <v>46043</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" t="s">
         <v>39</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>40</v>
       </c>
-      <c r="F18" t="s">
-        <v>41</v>
-      </c>
       <c r="G18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>11</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="4">
         <v>46043</v>
       </c>
       <c r="C19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" t="s">
         <v>42</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>43</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>44</v>
       </c>
-      <c r="F19" t="s">
-        <v>45</v>
-      </c>
       <c r="G19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>12</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="4">
         <v>46043</v>
       </c>
       <c r="C20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" t="s">
         <v>46</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>47</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>48</v>
       </c>
-      <c r="F20" t="s">
-        <v>49</v>
-      </c>
       <c r="G20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>